<commit_message>
fix: uploading the new 2025 data / adding a new column 'prefix' for data after 2020 for the section ones
</commit_message>
<xml_diff>
--- a/data/raw_data/2025/permits-by-county-2025.xlsx
+++ b/data/raw_data/2025/permits-by-county-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naughtm\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32472976-728B-47BE-B0D0-539701595FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1721F508-B303-467E-8E86-C528D7E9550E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0804BE60-6E3F-46A7-BE5A-4D35DED6C4F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FF63E75D-8914-486B-9442-25E0E8AEBF27}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,91 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+  <si>
+    <t>Antrim</t>
+  </si>
+  <si>
+    <t>Carlow</t>
+  </si>
+  <si>
+    <t>Cavan</t>
+  </si>
+  <si>
+    <t>Clare</t>
+  </si>
+  <si>
+    <t>Cork</t>
+  </si>
+  <si>
+    <t>Donegal</t>
+  </si>
+  <si>
+    <t>Dublin</t>
+  </si>
+  <si>
+    <t>Galway</t>
+  </si>
+  <si>
+    <t>Kerry</t>
+  </si>
+  <si>
+    <t>Kildare</t>
+  </si>
+  <si>
+    <t>Kilkenny</t>
+  </si>
+  <si>
+    <t>Laois</t>
+  </si>
+  <si>
+    <t>Leitrim</t>
+  </si>
+  <si>
+    <t>Limerick</t>
+  </si>
+  <si>
+    <t>Longford</t>
+  </si>
+  <si>
+    <t>Louth</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Meath</t>
+  </si>
+  <si>
+    <t>Monaghan</t>
+  </si>
+  <si>
+    <t>Offaly</t>
+  </si>
+  <si>
+    <t>Roscommon</t>
+  </si>
+  <si>
+    <t>Sligo</t>
+  </si>
+  <si>
+    <t>Tipperary</t>
+  </si>
+  <si>
+    <t>Waterford</t>
+  </si>
+  <si>
+    <t>Westmeath</t>
+  </si>
+  <si>
+    <t>Wexford</t>
+  </si>
+  <si>
+    <t>Wicklow</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
   <si>
     <t>2025</t>
   </si>
@@ -45,99 +129,6 @@
   </si>
   <si>
     <t>Refused</t>
-  </si>
-  <si>
-    <t>Withdrawn</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>No County Entered</t>
-  </si>
-  <si>
-    <t>Antrim</t>
-  </si>
-  <si>
-    <t>Carlow</t>
-  </si>
-  <si>
-    <t>Cavan</t>
-  </si>
-  <si>
-    <t>Clare</t>
-  </si>
-  <si>
-    <t>Cork</t>
-  </si>
-  <si>
-    <t>Donegal</t>
-  </si>
-  <si>
-    <t>Down</t>
-  </si>
-  <si>
-    <t>Dublin</t>
-  </si>
-  <si>
-    <t>Galway</t>
-  </si>
-  <si>
-    <t>Kerry</t>
-  </si>
-  <si>
-    <t>Kildare</t>
-  </si>
-  <si>
-    <t>Kilkenny</t>
-  </si>
-  <si>
-    <t>Laois</t>
-  </si>
-  <si>
-    <t>Leitrim</t>
-  </si>
-  <si>
-    <t>Limerick</t>
-  </si>
-  <si>
-    <t>Longford</t>
-  </si>
-  <si>
-    <t>Louth</t>
-  </si>
-  <si>
-    <t>Mayo</t>
-  </si>
-  <si>
-    <t>Meath</t>
-  </si>
-  <si>
-    <t>Monaghan</t>
-  </si>
-  <si>
-    <t>Offaly</t>
-  </si>
-  <si>
-    <t>Roscommon</t>
-  </si>
-  <si>
-    <t>Sligo</t>
-  </si>
-  <si>
-    <t>Tipperary</t>
-  </si>
-  <si>
-    <t>Waterford</t>
-  </si>
-  <si>
-    <t>Westmeath</t>
-  </si>
-  <si>
-    <t>Wexford</t>
-  </si>
-  <si>
-    <t>Wicklow</t>
   </si>
 </sst>
 </file>
@@ -153,6 +144,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
@@ -160,14 +157,9 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFA20000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -207,28 +199,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,454 +548,346 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ADC3E56-DC3E-4CE3-9608-72F2228540D6}">
-  <dimension ref="A1:D32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DC6779-5101-470A-9A7D-9F3DE816E57B}">
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="5"/>
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="5"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="8">
+        <v>31044</v>
+      </c>
+      <c r="C3" s="8">
+        <v>3432</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3">
+        <v>181</v>
+      </c>
+      <c r="C5" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B6" s="3">
+        <v>501</v>
+      </c>
+      <c r="C6" s="3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B7" s="3">
+        <v>538</v>
+      </c>
+      <c r="C7" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8">
-        <v>22542</v>
-      </c>
-      <c r="C3" s="8">
-        <v>2421</v>
-      </c>
-      <c r="D3" s="8">
-        <v>13874</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B8" s="3">
+        <v>2973</v>
+      </c>
+      <c r="C8" s="3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="7">
-        <v>4620</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="B9" s="3">
+        <v>488</v>
+      </c>
+      <c r="C9" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7">
-        <v>1</v>
-      </c>
-      <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B10" s="3">
+        <v>14627</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1395</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="7">
-        <v>128</v>
-      </c>
-      <c r="C6" s="7">
+      <c r="B11" s="3">
+        <v>1104</v>
+      </c>
+      <c r="C11" s="3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3">
+        <v>527</v>
+      </c>
+      <c r="C12" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3">
+        <v>1194</v>
+      </c>
+      <c r="C13" s="3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3">
+        <v>580</v>
+      </c>
+      <c r="C14" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="3">
+        <v>229</v>
+      </c>
+      <c r="C15" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3">
+        <v>99</v>
+      </c>
+      <c r="C16" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="3">
+        <v>1543</v>
+      </c>
+      <c r="C17" s="3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="7">
-        <v>385</v>
-      </c>
-      <c r="C7" s="7">
+      <c r="B18" s="3">
+        <v>147</v>
+      </c>
+      <c r="C18" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3">
+        <v>511</v>
+      </c>
+      <c r="C19" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3">
+        <v>383</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="3">
+        <v>1252</v>
+      </c>
+      <c r="C21" s="3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3">
+        <v>449</v>
+      </c>
+      <c r="C22" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="3">
+        <v>358</v>
+      </c>
+      <c r="C23" s="3">
         <v>40</v>
       </c>
-      <c r="D7" s="7">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="7">
-        <v>379</v>
-      </c>
-      <c r="C8" s="7">
-        <v>54</v>
-      </c>
-      <c r="D8" s="7">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="7">
-        <v>2130</v>
-      </c>
-      <c r="C9" s="7">
-        <v>224</v>
-      </c>
-      <c r="D9" s="7">
-        <v>898</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="7">
-        <v>377</v>
-      </c>
-      <c r="C10" s="7">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3">
+        <v>188</v>
+      </c>
+      <c r="C24" s="3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="3">
+        <v>218</v>
+      </c>
+      <c r="C25" s="3">
         <v>52</v>
       </c>
-      <c r="D10" s="7">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="7">
-        <v>1</v>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="7">
-        <v>10503</v>
-      </c>
-      <c r="C12" s="7">
-        <v>997</v>
-      </c>
-      <c r="D12" s="7">
-        <v>3715</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="7">
-        <v>765</v>
-      </c>
-      <c r="C13" s="7">
-        <v>85</v>
-      </c>
-      <c r="D13" s="7">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="7">
-        <v>396</v>
-      </c>
-      <c r="C14" s="7">
-        <v>38</v>
-      </c>
-      <c r="D14" s="7">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="7">
-        <v>914</v>
-      </c>
-      <c r="C15" s="7">
-        <v>139</v>
-      </c>
-      <c r="D15" s="7">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="7">
-        <v>405</v>
-      </c>
-      <c r="C16" s="7">
-        <v>33</v>
-      </c>
-      <c r="D16" s="7">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="7">
-        <v>170</v>
-      </c>
-      <c r="C17" s="7">
-        <v>50</v>
-      </c>
-      <c r="D17" s="7">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="7">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3">
+        <v>650</v>
+      </c>
+      <c r="C26" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="3">
+        <v>695</v>
+      </c>
+      <c r="C27" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3">
+        <v>457</v>
+      </c>
+      <c r="C28" s="3">
         <v>68</v>
       </c>
-      <c r="C18" s="7">
-        <v>6</v>
-      </c>
-      <c r="D18" s="7">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="3">
+        <v>762</v>
+      </c>
+      <c r="C29" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="7">
-        <v>1164</v>
-      </c>
-      <c r="C19" s="7">
-        <v>123</v>
-      </c>
-      <c r="D19" s="7">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="7">
-        <v>101</v>
-      </c>
-      <c r="C20" s="7">
-        <v>17</v>
-      </c>
-      <c r="D20" s="7">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="7">
-        <v>348</v>
-      </c>
-      <c r="C21" s="7">
-        <v>35</v>
-      </c>
-      <c r="D21" s="7">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="7">
-        <v>271</v>
-      </c>
-      <c r="C22" s="7">
-        <v>33</v>
-      </c>
-      <c r="D22" s="7">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="7">
-        <v>907</v>
-      </c>
-      <c r="C23" s="7">
-        <v>146</v>
-      </c>
-      <c r="D23" s="7">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="7">
-        <v>351</v>
-      </c>
-      <c r="C24" s="7">
-        <v>29</v>
-      </c>
-      <c r="D24" s="7">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="7">
-        <v>268</v>
-      </c>
-      <c r="C25" s="7">
-        <v>23</v>
-      </c>
-      <c r="D25" s="7">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="7">
-        <v>141</v>
-      </c>
-      <c r="C26" s="7">
-        <v>19</v>
-      </c>
-      <c r="D26" s="7">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="7">
-        <v>158</v>
-      </c>
-      <c r="C27" s="7">
-        <v>38</v>
-      </c>
-      <c r="D27" s="7">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="7">
-        <v>491</v>
-      </c>
-      <c r="C28" s="7">
-        <v>43</v>
-      </c>
-      <c r="D28" s="7">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="7">
-        <v>566</v>
-      </c>
-      <c r="C29" s="7">
-        <v>55</v>
-      </c>
-      <c r="D29" s="7">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="7">
-        <v>315</v>
-      </c>
-      <c r="C30" s="7">
-        <v>59</v>
-      </c>
-      <c r="D30" s="7">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="7">
-        <v>565</v>
-      </c>
-      <c r="C31" s="7">
-        <v>41</v>
-      </c>
-      <c r="D31" s="7">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="7">
-        <v>275</v>
-      </c>
-      <c r="C32" s="7">
-        <v>27</v>
-      </c>
-      <c r="D32" s="7">
-        <v>171</v>
+      <c r="B30" s="3">
+        <v>390</v>
+      </c>
+      <c r="C30" s="3">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="eDocument" ma:contentTypeID="0x0101000BC94875665D404BB1351B53C41FD2C000E5CBA74D75A77049B177D97877D56E03" ma:contentTypeVersion="181" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="9aef13b51d858ac71ab25d278c7edb31">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f94102a1-1d6c-4502-ac27-91905b9321dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="992d5dd0ba35d17e896caa4d336a12f8" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="eDocument" ma:contentTypeID="0x0101000BC94875665D404BB1351B53C41FD2C000E5CBA74D75A77049B177D97877D56E03" ma:contentTypeVersion="199" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="f29b0ff1a26a7575c948acee1be83c00">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f94102a1-1d6c-4502-ac27-91905b9321dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3fe347a261331acec84421138fd81903" ns2:_="">
     <xsd:import namespace="f94102a1-1d6c-4502-ac27-91905b9321dd"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -1265,7 +1143,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8906BC1-B9F8-468F-B62B-D526A3815BEC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{994080F9-4AE5-42D2-83A1-83F2215EFC23}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1283,14 +1161,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B9E62FD8-E82F-4E04-9CFE-AF6725E34E21}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4AC580B-C109-4393-9C55-DCF18D6B72BD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="f94102a1-1d6c-4502-ac27-91905b9321dd"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -1299,7 +1177,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED1DE1DA-BB70-4DB0-810A-3DCE6B3A632C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F2F7CC-751F-4459-A1A8-B354A133568A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>

</xml_diff>